<commit_message>
fixed some more changes in default risk assessment
</commit_message>
<xml_diff>
--- a/Audit_Code/public/assets_template.xlsx
+++ b/Audit_Code/public/assets_template.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ab\Desktop\Compliance\Audit_Code\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhammad.abdullah\Documents\Compliance\Audit_Code\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9630"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9636"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,9 +26,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
-    <t>Asset Group Name</t>
-  </si>
-  <si>
     <t>Asset Component Name</t>
   </si>
   <si>
@@ -44,7 +41,10 @@
     <t>Service Name</t>
   </si>
   <si>
-    <t>Asset  Name</t>
+    <t>Asset Type</t>
+  </si>
+  <si>
+    <t>Asset Subtype</t>
   </si>
 </sst>
 </file>
@@ -363,38 +363,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" customWidth="1"/>
-    <col min="3" max="3" width="23.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17.140625" customWidth="1"/>
-    <col min="5" max="5" width="22.5703125" customWidth="1"/>
-    <col min="6" max="6" width="23.42578125" customWidth="1"/>
-    <col min="7" max="7" width="41.5703125" customWidth="1"/>
+    <col min="1" max="1" width="24.33203125" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
+    <col min="3" max="3" width="23.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.109375" customWidth="1"/>
+    <col min="5" max="5" width="22.5546875" customWidth="1"/>
+    <col min="6" max="6" width="23.44140625" customWidth="1"/>
+    <col min="7" max="7" width="41.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
         <v>5</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
       </c>
       <c r="C1" t="s">
         <v>6</v>
       </c>
       <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed changes for owner dept
</commit_message>
<xml_diff>
--- a/Audit_Code/public/assets_template.xlsx
+++ b/Audit_Code/public/assets_template.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhammad.abdullah\Documents\Compliance\Audit_Code\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Compliance\Audit_Code\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9636"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9630"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,12 +24,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Asset Component Name</t>
-  </si>
-  <si>
-    <t>Asset Owner Dept.</t>
   </si>
   <si>
     <t>Asset Physical Location</t>
@@ -50,7 +47,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -362,27 +359,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.33203125" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" customWidth="1"/>
-    <col min="3" max="3" width="23.6640625" customWidth="1"/>
-    <col min="4" max="4" width="17.109375" customWidth="1"/>
-    <col min="5" max="5" width="22.5546875" customWidth="1"/>
-    <col min="6" max="6" width="23.44140625" customWidth="1"/>
-    <col min="7" max="7" width="41.5546875" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="6" max="6" width="41.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
@@ -392,9 +388,6 @@
       </c>
       <c r="F1" t="s">
         <v>2</v>
-      </c>
-      <c r="G1" t="s">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>